<commit_message>
docs: update dataset spreadsheet columns
</commit_message>
<xml_diff>
--- a/spreadsheet/linear_regression_dataset_spreadsheet.xlsx
+++ b/spreadsheet/linear_regression_dataset_spreadsheet.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,13 +28,25 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <color theme="10"/>
+      <sz val="12"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -52,17 +64,26 @@
       <bottom style="thin"/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -425,537 +446,710 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:I21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="72" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="88" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Nama</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>NIM</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Kelas</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Recommendation</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>Source URL</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Recommended Target</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Deskripsi Singkat</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr"/>
+      <c r="C2" s="3" t="inlineStr"/>
+      <c r="D2" s="3" t="inlineStr"/>
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t>Concrete Compressive Strength</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="F2" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/165/concrete+compressive+strength</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Concrete compressive strength</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi kuat tekan beton dari komposisi bahan dan umur beton.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr"/>
+      <c r="C3" s="3" t="inlineStr"/>
+      <c r="D3" s="3" t="inlineStr"/>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Energy Efficiency</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="F3" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/242/energy+efficiency</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Heating Load or Cooling Load</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi beban pemanasan atau pendinginan bangunan dari fitur desain bangunan.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr"/>
+      <c r="C4" s="3" t="inlineStr"/>
+      <c r="D4" s="3" t="inlineStr"/>
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Real Estate Valuation</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="F4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/477/real+estate+valuation+data+set</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>house price of unit area</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi harga rumah per unit area dari fitur lokasi dan properti.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr"/>
+      <c r="C5" s="3" t="inlineStr"/>
+      <c r="D5" s="3" t="inlineStr"/>
+      <c r="E5" s="3" t="inlineStr">
         <is>
           <t>Auto MPG</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="F5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/9/auto+mpg</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="H5" s="3" t="inlineStr">
         <is>
           <t>mpg</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi efisiensi bahan bakar mobil dalam MPG dari spesifikasi kendaraan.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr"/>
+      <c r="C6" s="3" t="inlineStr"/>
+      <c r="D6" s="3" t="inlineStr"/>
+      <c r="E6" s="3" t="inlineStr">
         <is>
           <t>Combined Cycle Power Plant</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="F6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/294/combined+cycle+power+plant</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>PE</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi output energi pembangkit listrik dari kondisi lingkungan.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="3" t="n">
         <v>6</v>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr"/>
+      <c r="C7" s="3" t="inlineStr"/>
+      <c r="D7" s="3" t="inlineStr"/>
+      <c r="E7" s="3" t="inlineStr">
         <is>
           <t>Bike Sharing Dataset</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="F7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/275/bike+sharing+dataset</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="H7" s="3" t="inlineStr">
         <is>
           <t>cnt</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi jumlah penyewaan sepeda dari informasi cuaca dan waktu.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr"/>
+      <c r="C8" s="3" t="inlineStr"/>
+      <c r="D8" s="3" t="inlineStr"/>
+      <c r="E8" s="3" t="inlineStr">
         <is>
           <t>Wine Quality</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="F8" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G8" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/186/wine+quality</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>quality</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi kualitas wine dari fitur kimia yang semuanya numerik.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr"/>
+      <c r="C9" s="3" t="inlineStr"/>
+      <c r="D9" s="3" t="inlineStr"/>
+      <c r="E9" s="3" t="inlineStr">
         <is>
           <t>Student Performance</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="F9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/320/student+performance</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="H9" s="3" t="inlineStr">
         <is>
           <t>G3</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi nilai akhir siswa dari data akademik dan karakteristik siswa.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr"/>
+      <c r="C10" s="3" t="inlineStr"/>
+      <c r="D10" s="3" t="inlineStr"/>
+      <c r="E10" s="3" t="inlineStr">
         <is>
           <t>Air Quality</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="F10" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/360/air+quality</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>CO(GT) or NOx(GT) or NO2(GT)</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI sensor kualitas udara untuk memprediksi konsentrasi polutan numerik.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr"/>
+      <c r="C11" s="3" t="inlineStr"/>
+      <c r="D11" s="3" t="inlineStr"/>
+      <c r="E11" s="3" t="inlineStr">
         <is>
           <t>Medical Cost Personal Dataset / Insurance</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="F11" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G11" s="4" t="inlineStr">
         <is>
           <t>https://www.kaggle.com/datasets/mirichoi0218/insurance</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>charges</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>Dataset Kaggle untuk memprediksi biaya asuransi kesehatan dari data demografi dan kebiasaan.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr"/>
+      <c r="E12" s="3" t="inlineStr">
         <is>
           <t>Fish Market</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="F12" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
         <is>
           <t>https://www.kaggle.com/datasets/vipullrathod/fish-market</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t>Dataset Kaggle untuk memprediksi berat ikan dari ukuran fisik dan spesies ikan.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B13" s="3" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr"/>
+      <c r="D13" s="3" t="inlineStr"/>
+      <c r="E13" s="3" t="inlineStr">
         <is>
           <t>Seoul Bike Sharing Demand</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="F13" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G13" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/560/seoul+bike+sharing+demand</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>Rented Bike Count</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi jumlah penyewaan sepeda di Seoul dari cuaca dan kalender.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="3" t="n">
         <v>13</v>
       </c>
-      <c r="B14" t="inlineStr">
+      <c r="B14" s="3" t="inlineStr"/>
+      <c r="C14" s="3" t="inlineStr"/>
+      <c r="D14" s="3" t="inlineStr"/>
+      <c r="E14" s="3" t="inlineStr">
         <is>
           <t>House Rent Prediction Dataset</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr">
+      <c r="F14" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" s="4" t="inlineStr">
         <is>
           <t>https://www.kaggle.com/datasets/iamsouravbanerjee/house-rent-prediction-dataset</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>Rent</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr">
+      <c r="I14" s="3" t="inlineStr">
         <is>
           <t>Dataset Kaggle untuk memprediksi harga sewa rumah dari lokasi dan detail properti.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="3" t="n">
         <v>14</v>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr"/>
+      <c r="C15" s="3" t="inlineStr"/>
+      <c r="D15" s="3" t="inlineStr"/>
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>Airfoil Self-Noise</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
+      <c r="F15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/291/airfoil+self+noise</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr">
+      <c r="H15" s="3" t="inlineStr">
         <is>
           <t>scaled-sound-pressure</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr">
+      <c r="I15" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI eksperimen airfoil NASA untuk memprediksi tingkat tekanan suara.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr"/>
+      <c r="C16" s="3" t="inlineStr"/>
+      <c r="D16" s="3" t="inlineStr"/>
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>Yacht Hydrodynamics</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="F16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G16" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/ml/datasets/yacht+hydrodynamics</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>residuary resistance</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="I16" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi hambatan residu yacht dari parameter hidrodinamika.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="3" t="n">
         <v>16</v>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B17" s="3" t="inlineStr"/>
+      <c r="C17" s="3" t="inlineStr"/>
+      <c r="D17" s="3" t="inlineStr"/>
+      <c r="E17" s="3" t="inlineStr">
         <is>
           <t>Appliances Energy Prediction</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="F17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/374/appliances+energy+prediction</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="H17" s="3" t="inlineStr">
         <is>
           <t>Appliances</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="I17" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi konsumsi energi peralatan rumah dari data suhu, kelembapan, dan waktu.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="3" t="n">
         <v>17</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="3" t="inlineStr"/>
+      <c r="C18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr"/>
+      <c r="E18" s="3" t="inlineStr">
         <is>
           <t>Concrete Slump Test</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="F18" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/182/concrete+slump+test</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>Compressive Strength or SLUMP or FLOW</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="I18" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI beton slump untuk memprediksi kekuatan tekan atau karakteristik beton segar.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="3" t="n">
         <v>18</v>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="B19" s="3" t="inlineStr"/>
+      <c r="C19" s="3" t="inlineStr"/>
+      <c r="D19" s="3" t="inlineStr"/>
+      <c r="E19" s="3" t="inlineStr">
         <is>
           <t>Computer Hardware</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr">
+      <c r="F19" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="G19" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/ml/datasets/computer+hardware</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
+      <c r="H19" s="3" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr">
+      <c r="I19" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi performa CPU dari spesifikasi perangkat keras komputer.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="3" t="n">
         <v>19</v>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="3" t="inlineStr"/>
+      <c r="C20" s="3" t="inlineStr"/>
+      <c r="D20" s="3" t="inlineStr"/>
+      <c r="E20" s="3" t="inlineStr">
         <is>
           <t>QSAR Fish Toxicity</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="F20" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/504/qsar+fish+toxicity</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>LC50</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="I20" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI kimia untuk memprediksi toksisitas ikan dari fitur molekuler numerik.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr"/>
+      <c r="C21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr"/>
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>Abalone</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="F21" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/1/abalone</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="H21" s="3" t="inlineStr">
         <is>
           <t>Rings</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="I21" s="3" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi jumlah rings abalone dari ukuran fisik dan jenis kelamin.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: split dataset list and submissions sheets
</commit_message>
<xml_diff>
--- a/spreadsheet/linear_regression_dataset_spreadsheet.xlsx
+++ b/spreadsheet/linear_regression_dataset_spreadsheet.xlsx
@@ -7,9 +7,13 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dataset" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="List Dataset" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pengumpulan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'List Dataset'!$A$1:$F$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pengumpulan'!$A$1:$G$101</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -36,7 +40,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -48,20 +52,19 @@
         <fgColor rgb="00D9EAF7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="2">
@@ -70,16 +73,16 @@
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -446,710 +449,1799 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="72" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="88" customWidth="1" min="9" max="9"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="88" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Nama</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>NIM</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Kelas</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Dataset</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Recommendation</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Source URL</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Target</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Deskripsi Singkat</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="n">
+      <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="inlineStr"/>
-      <c r="C2" s="3" t="inlineStr"/>
-      <c r="D2" s="3" t="inlineStr"/>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>Concrete Compressive Strength</t>
         </is>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="C2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/165/concrete+compressive+strength</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Concrete compressive strength</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi kuat tekan beton dari komposisi bahan dan umur beton.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="n">
+      <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="3" t="inlineStr"/>
-      <c r="C3" s="3" t="inlineStr"/>
-      <c r="D3" s="3" t="inlineStr"/>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>Energy Efficiency</t>
         </is>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="C3" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/242/energy+efficiency</t>
         </is>
       </c>
-      <c r="H3" s="3" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Heating Load or Cooling Load</t>
         </is>
       </c>
-      <c r="I3" s="3" t="inlineStr">
+      <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi beban pemanasan atau pendinginan bangunan dari fitur desain bangunan.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="n">
+      <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="3" t="inlineStr"/>
-      <c r="C4" s="3" t="inlineStr"/>
-      <c r="D4" s="3" t="inlineStr"/>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>Real Estate Valuation</t>
         </is>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="C4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/477/real+estate+valuation+data+set</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>house price of unit area</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi harga rumah per unit area dari fitur lokasi dan properti.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="n">
+      <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="3" t="inlineStr"/>
-      <c r="C5" s="3" t="inlineStr"/>
-      <c r="D5" s="3" t="inlineStr"/>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>Auto MPG</t>
         </is>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="C5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/9/auto+mpg</t>
         </is>
       </c>
-      <c r="H5" s="3" t="inlineStr">
+      <c r="E5" s="2" t="inlineStr">
         <is>
           <t>mpg</t>
         </is>
       </c>
-      <c r="I5" s="3" t="inlineStr">
+      <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi efisiensi bahan bakar mobil dalam MPG dari spesifikasi kendaraan.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="n">
+      <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="3" t="inlineStr"/>
-      <c r="C6" s="3" t="inlineStr"/>
-      <c r="D6" s="3" t="inlineStr"/>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Combined Cycle Power Plant</t>
         </is>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="C6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/294/combined+cycle+power+plant</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>PE</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi output energi pembangkit listrik dari kondisi lingkungan.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="n">
+      <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="3" t="inlineStr"/>
-      <c r="C7" s="3" t="inlineStr"/>
-      <c r="D7" s="3" t="inlineStr"/>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>Bike Sharing Dataset</t>
         </is>
       </c>
-      <c r="F7" s="3" t="n">
+      <c r="C7" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/275/bike+sharing+dataset</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="E7" s="2" t="inlineStr">
         <is>
           <t>cnt</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi jumlah penyewaan sepeda dari informasi cuaca dan waktu.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="n">
+      <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="3" t="inlineStr"/>
-      <c r="C8" s="3" t="inlineStr"/>
-      <c r="D8" s="3" t="inlineStr"/>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Wine Quality</t>
         </is>
       </c>
-      <c r="F8" s="3" t="n">
+      <c r="C8" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/186/wine+quality</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>quality</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi kualitas wine dari fitur kimia yang semuanya numerik.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="n">
+      <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="3" t="inlineStr"/>
-      <c r="C9" s="3" t="inlineStr"/>
-      <c r="D9" s="3" t="inlineStr"/>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="B9" s="2" t="inlineStr">
         <is>
           <t>Student Performance</t>
         </is>
       </c>
-      <c r="F9" s="3" t="n">
+      <c r="C9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/320/student+performance</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr">
+      <c r="E9" s="2" t="inlineStr">
         <is>
           <t>G3</t>
         </is>
       </c>
-      <c r="I9" s="3" t="inlineStr">
+      <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi nilai akhir siswa dari data akademik dan karakteristik siswa.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="n">
+      <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="3" t="inlineStr"/>
-      <c r="C10" s="3" t="inlineStr"/>
-      <c r="D10" s="3" t="inlineStr"/>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="B10" s="2" t="inlineStr">
         <is>
           <t>Air Quality</t>
         </is>
       </c>
-      <c r="F10" s="3" t="n">
+      <c r="C10" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G10" s="4" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/360/air+quality</t>
         </is>
       </c>
-      <c r="H10" s="3" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>CO(GT) or NOx(GT) or NO2(GT)</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI sensor kualitas udara untuk memprediksi konsentrasi polutan numerik.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="n">
+      <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="3" t="inlineStr"/>
-      <c r="C11" s="3" t="inlineStr"/>
-      <c r="D11" s="3" t="inlineStr"/>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="B11" s="2" t="inlineStr">
         <is>
           <t>Medical Cost Personal Dataset / Insurance</t>
         </is>
       </c>
-      <c r="F11" s="3" t="n">
+      <c r="C11" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t>https://www.kaggle.com/datasets/mirichoi0218/insurance</t>
         </is>
       </c>
-      <c r="H11" s="3" t="inlineStr">
+      <c r="E11" s="2" t="inlineStr">
         <is>
           <t>charges</t>
         </is>
       </c>
-      <c r="I11" s="3" t="inlineStr">
+      <c r="F11" s="2" t="inlineStr">
         <is>
           <t>Dataset Kaggle untuk memprediksi biaya asuransi kesehatan dari data demografi dan kebiasaan.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n">
+      <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="3" t="inlineStr"/>
-      <c r="C12" s="3" t="inlineStr"/>
-      <c r="D12" s="3" t="inlineStr"/>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="B12" s="2" t="inlineStr">
         <is>
           <t>Fish Market</t>
         </is>
       </c>
-      <c r="F12" s="3" t="n">
+      <c r="C12" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>https://www.kaggle.com/datasets/vipullrathod/fish-market</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>Dataset Kaggle untuk memprediksi berat ikan dari ukuran fisik dan spesies ikan.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="n">
+      <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="3" t="inlineStr"/>
-      <c r="C13" s="3" t="inlineStr"/>
-      <c r="D13" s="3" t="inlineStr"/>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="B13" s="2" t="inlineStr">
         <is>
           <t>Seoul Bike Sharing Demand</t>
         </is>
       </c>
-      <c r="F13" s="3" t="n">
+      <c r="C13" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="D13" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/560/seoul+bike+sharing+demand</t>
         </is>
       </c>
-      <c r="H13" s="3" t="inlineStr">
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>Rented Bike Count</t>
         </is>
       </c>
-      <c r="I13" s="3" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi jumlah penyewaan sepeda di Seoul dari cuaca dan kalender.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="n">
+      <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr"/>
-      <c r="C14" s="3" t="inlineStr"/>
-      <c r="D14" s="3" t="inlineStr"/>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
         <is>
           <t>House Rent Prediction Dataset</t>
         </is>
       </c>
-      <c r="F14" s="3" t="n">
+      <c r="C14" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="D14" s="3" t="inlineStr">
         <is>
           <t>https://www.kaggle.com/datasets/iamsouravbanerjee/house-rent-prediction-dataset</t>
         </is>
       </c>
-      <c r="H14" s="3" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Rent</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>Dataset Kaggle untuk memprediksi harga sewa rumah dari lokasi dan detail properti.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="n">
+      <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="3" t="inlineStr"/>
-      <c r="C15" s="3" t="inlineStr"/>
-      <c r="D15" s="3" t="inlineStr"/>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>Airfoil Self-Noise</t>
         </is>
       </c>
-      <c r="F15" s="3" t="n">
+      <c r="C15" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/291/airfoil+self+noise</t>
         </is>
       </c>
-      <c r="H15" s="3" t="inlineStr">
+      <c r="E15" s="2" t="inlineStr">
         <is>
           <t>scaled-sound-pressure</t>
         </is>
       </c>
-      <c r="I15" s="3" t="inlineStr">
+      <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI eksperimen airfoil NASA untuk memprediksi tingkat tekanan suara.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="n">
+      <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="3" t="inlineStr"/>
-      <c r="C16" s="3" t="inlineStr"/>
-      <c r="D16" s="3" t="inlineStr"/>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>Yacht Hydrodynamics</t>
         </is>
       </c>
-      <c r="F16" s="3" t="n">
+      <c r="C16" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G16" s="4" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/ml/datasets/yacht+hydrodynamics</t>
         </is>
       </c>
-      <c r="H16" s="3" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>residuary resistance</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi hambatan residu yacht dari parameter hidrodinamika.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="n">
+      <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="3" t="inlineStr"/>
-      <c r="C17" s="3" t="inlineStr"/>
-      <c r="D17" s="3" t="inlineStr"/>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="B17" s="2" t="inlineStr">
         <is>
           <t>Appliances Energy Prediction</t>
         </is>
       </c>
-      <c r="F17" s="3" t="n">
+      <c r="C17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="D17" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/374/appliances+energy+prediction</t>
         </is>
       </c>
-      <c r="H17" s="3" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Appliances</t>
         </is>
       </c>
-      <c r="I17" s="3" t="inlineStr">
+      <c r="F17" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi konsumsi energi peralatan rumah dari data suhu, kelembapan, dan waktu.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="n">
+      <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="3" t="inlineStr"/>
-      <c r="C18" s="3" t="inlineStr"/>
-      <c r="D18" s="3" t="inlineStr"/>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Concrete Slump Test</t>
         </is>
       </c>
-      <c r="F18" s="3" t="n">
+      <c r="C18" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="G18" s="4" t="inlineStr">
+      <c r="D18" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/182/concrete+slump+test</t>
         </is>
       </c>
-      <c r="H18" s="3" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Compressive Strength or SLUMP or FLOW</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI beton slump untuk memprediksi kekuatan tekan atau karakteristik beton segar.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="n">
+      <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="3" t="inlineStr"/>
-      <c r="C19" s="3" t="inlineStr"/>
-      <c r="D19" s="3" t="inlineStr"/>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>Computer Hardware</t>
         </is>
       </c>
-      <c r="F19" s="3" t="n">
+      <c r="C19" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="D19" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/ml/datasets/computer+hardware</t>
         </is>
       </c>
-      <c r="H19" s="3" t="inlineStr">
+      <c r="E19" s="2" t="inlineStr">
         <is>
           <t>PRP</t>
         </is>
       </c>
-      <c r="I19" s="3" t="inlineStr">
+      <c r="F19" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi performa CPU dari spesifikasi perangkat keras komputer.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="n">
+      <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="3" t="inlineStr"/>
-      <c r="C20" s="3" t="inlineStr"/>
-      <c r="D20" s="3" t="inlineStr"/>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>QSAR Fish Toxicity</t>
         </is>
       </c>
-      <c r="F20" s="3" t="n">
+      <c r="C20" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="D20" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/504/qsar+fish+toxicity</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>LC50</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI kimia untuk memprediksi toksisitas ikan dari fitur molekuler numerik.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="n">
+      <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="3" t="inlineStr"/>
-      <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>Abalone</t>
         </is>
       </c>
-      <c r="F21" s="3" t="n">
+      <c r="C21" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="D21" s="3" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/1/abalone</t>
         </is>
       </c>
-      <c r="H21" s="3" t="inlineStr">
+      <c r="E21" s="2" t="inlineStr">
         <is>
           <t>Rings</t>
         </is>
       </c>
-      <c r="I21" s="3" t="inlineStr">
+      <c r="F21" s="2" t="inlineStr">
         <is>
           <t>Dataset UCI untuk memprediksi jumlah rings abalone dari ukuran fisik dan jenis kelamin.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:F21"/>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G11" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G12" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G13" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G14" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G15" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G16" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G17" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G18" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G19" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G20" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId20"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G101"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="54" customWidth="1" min="6" max="6"/>
+    <col width="54" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>Nama</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>NIM</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>Kelas</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Dataset Yang Diambil</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Link Notebook Colab Shared</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Link Pengumpulan Peserta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr"/>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr"/>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr"/>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr"/>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr"/>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr"/>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr"/>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr"/>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr"/>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="2" t="inlineStr"/>
+      <c r="C12" s="2" t="inlineStr"/>
+      <c r="D12" s="2" t="inlineStr"/>
+      <c r="E12" s="2" t="inlineStr"/>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="2" t="inlineStr"/>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr"/>
+      <c r="E13" s="2" t="inlineStr"/>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="2" t="inlineStr"/>
+      <c r="C14" s="2" t="inlineStr"/>
+      <c r="D14" s="2" t="inlineStr"/>
+      <c r="E14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="2" t="inlineStr"/>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr"/>
+      <c r="E15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="2" t="inlineStr"/>
+      <c r="C16" s="2" t="inlineStr"/>
+      <c r="D16" s="2" t="inlineStr"/>
+      <c r="E16" s="2" t="inlineStr"/>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="2" t="inlineStr"/>
+      <c r="C17" s="2" t="inlineStr"/>
+      <c r="D17" s="2" t="inlineStr"/>
+      <c r="E17" s="2" t="inlineStr"/>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="2" t="inlineStr"/>
+      <c r="C18" s="2" t="inlineStr"/>
+      <c r="D18" s="2" t="inlineStr"/>
+      <c r="E18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr"/>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="2" t="inlineStr"/>
+      <c r="C20" s="2" t="inlineStr"/>
+      <c r="D20" s="2" t="inlineStr"/>
+      <c r="E20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="2" t="inlineStr"/>
+      <c r="C21" s="2" t="inlineStr"/>
+      <c r="D21" s="2" t="inlineStr"/>
+      <c r="E21" s="2" t="inlineStr"/>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="2" t="inlineStr"/>
+      <c r="C22" s="2" t="inlineStr"/>
+      <c r="D22" s="2" t="inlineStr"/>
+      <c r="E22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr"/>
+      <c r="G22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="2" t="inlineStr"/>
+      <c r="C23" s="2" t="inlineStr"/>
+      <c r="D23" s="2" t="inlineStr"/>
+      <c r="E23" s="2" t="inlineStr"/>
+      <c r="F23" s="2" t="inlineStr"/>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="2" t="inlineStr"/>
+      <c r="C24" s="2" t="inlineStr"/>
+      <c r="D24" s="2" t="inlineStr"/>
+      <c r="E24" s="2" t="inlineStr"/>
+      <c r="F24" s="2" t="inlineStr"/>
+      <c r="G24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="2" t="inlineStr"/>
+      <c r="C25" s="2" t="inlineStr"/>
+      <c r="D25" s="2" t="inlineStr"/>
+      <c r="E25" s="2" t="inlineStr"/>
+      <c r="F25" s="2" t="inlineStr"/>
+      <c r="G25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="2" t="inlineStr"/>
+      <c r="C26" s="2" t="inlineStr"/>
+      <c r="D26" s="2" t="inlineStr"/>
+      <c r="E26" s="2" t="inlineStr"/>
+      <c r="F26" s="2" t="inlineStr"/>
+      <c r="G26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="2" t="inlineStr"/>
+      <c r="C27" s="2" t="inlineStr"/>
+      <c r="D27" s="2" t="inlineStr"/>
+      <c r="E27" s="2" t="inlineStr"/>
+      <c r="F27" s="2" t="inlineStr"/>
+      <c r="G27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="2" t="inlineStr"/>
+      <c r="C28" s="2" t="inlineStr"/>
+      <c r="D28" s="2" t="inlineStr"/>
+      <c r="E28" s="2" t="inlineStr"/>
+      <c r="F28" s="2" t="inlineStr"/>
+      <c r="G28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="2" t="inlineStr"/>
+      <c r="C29" s="2" t="inlineStr"/>
+      <c r="D29" s="2" t="inlineStr"/>
+      <c r="E29" s="2" t="inlineStr"/>
+      <c r="F29" s="2" t="inlineStr"/>
+      <c r="G29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="2" t="inlineStr"/>
+      <c r="C30" s="2" t="inlineStr"/>
+      <c r="D30" s="2" t="inlineStr"/>
+      <c r="E30" s="2" t="inlineStr"/>
+      <c r="F30" s="2" t="inlineStr"/>
+      <c r="G30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="2" t="inlineStr"/>
+      <c r="C31" s="2" t="inlineStr"/>
+      <c r="D31" s="2" t="inlineStr"/>
+      <c r="E31" s="2" t="inlineStr"/>
+      <c r="F31" s="2" t="inlineStr"/>
+      <c r="G31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="2" t="inlineStr"/>
+      <c r="C32" s="2" t="inlineStr"/>
+      <c r="D32" s="2" t="inlineStr"/>
+      <c r="E32" s="2" t="inlineStr"/>
+      <c r="F32" s="2" t="inlineStr"/>
+      <c r="G32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="2" t="inlineStr"/>
+      <c r="C33" s="2" t="inlineStr"/>
+      <c r="D33" s="2" t="inlineStr"/>
+      <c r="E33" s="2" t="inlineStr"/>
+      <c r="F33" s="2" t="inlineStr"/>
+      <c r="G33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="2" t="inlineStr"/>
+      <c r="C34" s="2" t="inlineStr"/>
+      <c r="D34" s="2" t="inlineStr"/>
+      <c r="E34" s="2" t="inlineStr"/>
+      <c r="F34" s="2" t="inlineStr"/>
+      <c r="G34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="2" t="inlineStr"/>
+      <c r="C35" s="2" t="inlineStr"/>
+      <c r="D35" s="2" t="inlineStr"/>
+      <c r="E35" s="2" t="inlineStr"/>
+      <c r="F35" s="2" t="inlineStr"/>
+      <c r="G35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="2" t="inlineStr"/>
+      <c r="C36" s="2" t="inlineStr"/>
+      <c r="D36" s="2" t="inlineStr"/>
+      <c r="E36" s="2" t="inlineStr"/>
+      <c r="F36" s="2" t="inlineStr"/>
+      <c r="G36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="2" t="inlineStr"/>
+      <c r="C37" s="2" t="inlineStr"/>
+      <c r="D37" s="2" t="inlineStr"/>
+      <c r="E37" s="2" t="inlineStr"/>
+      <c r="F37" s="2" t="inlineStr"/>
+      <c r="G37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="2" t="inlineStr"/>
+      <c r="C38" s="2" t="inlineStr"/>
+      <c r="D38" s="2" t="inlineStr"/>
+      <c r="E38" s="2" t="inlineStr"/>
+      <c r="F38" s="2" t="inlineStr"/>
+      <c r="G38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="2" t="inlineStr"/>
+      <c r="C39" s="2" t="inlineStr"/>
+      <c r="D39" s="2" t="inlineStr"/>
+      <c r="E39" s="2" t="inlineStr"/>
+      <c r="F39" s="2" t="inlineStr"/>
+      <c r="G39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="2" t="inlineStr"/>
+      <c r="C40" s="2" t="inlineStr"/>
+      <c r="D40" s="2" t="inlineStr"/>
+      <c r="E40" s="2" t="inlineStr"/>
+      <c r="F40" s="2" t="inlineStr"/>
+      <c r="G40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="2" t="inlineStr"/>
+      <c r="C41" s="2" t="inlineStr"/>
+      <c r="D41" s="2" t="inlineStr"/>
+      <c r="E41" s="2" t="inlineStr"/>
+      <c r="F41" s="2" t="inlineStr"/>
+      <c r="G41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr"/>
+      <c r="D42" s="2" t="inlineStr"/>
+      <c r="E42" s="2" t="inlineStr"/>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="2" t="inlineStr"/>
+      <c r="C43" s="2" t="inlineStr"/>
+      <c r="D43" s="2" t="inlineStr"/>
+      <c r="E43" s="2" t="inlineStr"/>
+      <c r="F43" s="2" t="inlineStr"/>
+      <c r="G43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="2" t="inlineStr"/>
+      <c r="D44" s="2" t="inlineStr"/>
+      <c r="E44" s="2" t="inlineStr"/>
+      <c r="F44" s="2" t="inlineStr"/>
+      <c r="G44" s="2" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="2" t="inlineStr"/>
+      <c r="C45" s="2" t="inlineStr"/>
+      <c r="D45" s="2" t="inlineStr"/>
+      <c r="E45" s="2" t="inlineStr"/>
+      <c r="F45" s="2" t="inlineStr"/>
+      <c r="G45" s="2" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="2" t="inlineStr"/>
+      <c r="C46" s="2" t="inlineStr"/>
+      <c r="D46" s="2" t="inlineStr"/>
+      <c r="E46" s="2" t="inlineStr"/>
+      <c r="F46" s="2" t="inlineStr"/>
+      <c r="G46" s="2" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="2" t="inlineStr"/>
+      <c r="C47" s="2" t="inlineStr"/>
+      <c r="D47" s="2" t="inlineStr"/>
+      <c r="E47" s="2" t="inlineStr"/>
+      <c r="F47" s="2" t="inlineStr"/>
+      <c r="G47" s="2" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="2" t="inlineStr"/>
+      <c r="C48" s="2" t="inlineStr"/>
+      <c r="D48" s="2" t="inlineStr"/>
+      <c r="E48" s="2" t="inlineStr"/>
+      <c r="F48" s="2" t="inlineStr"/>
+      <c r="G48" s="2" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="2" t="inlineStr"/>
+      <c r="C49" s="2" t="inlineStr"/>
+      <c r="D49" s="2" t="inlineStr"/>
+      <c r="E49" s="2" t="inlineStr"/>
+      <c r="F49" s="2" t="inlineStr"/>
+      <c r="G49" s="2" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="2" t="inlineStr"/>
+      <c r="C50" s="2" t="inlineStr"/>
+      <c r="D50" s="2" t="inlineStr"/>
+      <c r="E50" s="2" t="inlineStr"/>
+      <c r="F50" s="2" t="inlineStr"/>
+      <c r="G50" s="2" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="2" t="inlineStr"/>
+      <c r="C51" s="2" t="inlineStr"/>
+      <c r="D51" s="2" t="inlineStr"/>
+      <c r="E51" s="2" t="inlineStr"/>
+      <c r="F51" s="2" t="inlineStr"/>
+      <c r="G51" s="2" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="2" t="inlineStr"/>
+      <c r="C52" s="2" t="inlineStr"/>
+      <c r="D52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr"/>
+      <c r="F52" s="2" t="inlineStr"/>
+      <c r="G52" s="2" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="2" t="inlineStr"/>
+      <c r="C53" s="2" t="inlineStr"/>
+      <c r="D53" s="2" t="inlineStr"/>
+      <c r="E53" s="2" t="inlineStr"/>
+      <c r="F53" s="2" t="inlineStr"/>
+      <c r="G53" s="2" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="2" t="inlineStr"/>
+      <c r="C54" s="2" t="inlineStr"/>
+      <c r="D54" s="2" t="inlineStr"/>
+      <c r="E54" s="2" t="inlineStr"/>
+      <c r="F54" s="2" t="inlineStr"/>
+      <c r="G54" s="2" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="2" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="2" t="inlineStr"/>
+      <c r="C55" s="2" t="inlineStr"/>
+      <c r="D55" s="2" t="inlineStr"/>
+      <c r="E55" s="2" t="inlineStr"/>
+      <c r="F55" s="2" t="inlineStr"/>
+      <c r="G55" s="2" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="2" t="inlineStr"/>
+      <c r="C56" s="2" t="inlineStr"/>
+      <c r="D56" s="2" t="inlineStr"/>
+      <c r="E56" s="2" t="inlineStr"/>
+      <c r="F56" s="2" t="inlineStr"/>
+      <c r="G56" s="2" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="2" t="inlineStr"/>
+      <c r="C57" s="2" t="inlineStr"/>
+      <c r="D57" s="2" t="inlineStr"/>
+      <c r="E57" s="2" t="inlineStr"/>
+      <c r="F57" s="2" t="inlineStr"/>
+      <c r="G57" s="2" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="2" t="inlineStr"/>
+      <c r="C58" s="2" t="inlineStr"/>
+      <c r="D58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr"/>
+      <c r="F58" s="2" t="inlineStr"/>
+      <c r="G58" s="2" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="2" t="inlineStr"/>
+      <c r="C59" s="2" t="inlineStr"/>
+      <c r="D59" s="2" t="inlineStr"/>
+      <c r="E59" s="2" t="inlineStr"/>
+      <c r="F59" s="2" t="inlineStr"/>
+      <c r="G59" s="2" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="2" t="inlineStr"/>
+      <c r="C60" s="2" t="inlineStr"/>
+      <c r="D60" s="2" t="inlineStr"/>
+      <c r="E60" s="2" t="inlineStr"/>
+      <c r="F60" s="2" t="inlineStr"/>
+      <c r="G60" s="2" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="2" t="inlineStr"/>
+      <c r="C61" s="2" t="inlineStr"/>
+      <c r="D61" s="2" t="inlineStr"/>
+      <c r="E61" s="2" t="inlineStr"/>
+      <c r="F61" s="2" t="inlineStr"/>
+      <c r="G61" s="2" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" s="2" t="inlineStr"/>
+      <c r="C62" s="2" t="inlineStr"/>
+      <c r="D62" s="2" t="inlineStr"/>
+      <c r="E62" s="2" t="inlineStr"/>
+      <c r="F62" s="2" t="inlineStr"/>
+      <c r="G62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" s="2" t="inlineStr"/>
+      <c r="C63" s="2" t="inlineStr"/>
+      <c r="D63" s="2" t="inlineStr"/>
+      <c r="E63" s="2" t="inlineStr"/>
+      <c r="F63" s="2" t="inlineStr"/>
+      <c r="G63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="2" t="inlineStr"/>
+      <c r="C64" s="2" t="inlineStr"/>
+      <c r="D64" s="2" t="inlineStr"/>
+      <c r="E64" s="2" t="inlineStr"/>
+      <c r="F64" s="2" t="inlineStr"/>
+      <c r="G64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="2" t="inlineStr"/>
+      <c r="C65" s="2" t="inlineStr"/>
+      <c r="D65" s="2" t="inlineStr"/>
+      <c r="E65" s="2" t="inlineStr"/>
+      <c r="F65" s="2" t="inlineStr"/>
+      <c r="G65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="2" t="inlineStr"/>
+      <c r="C66" s="2" t="inlineStr"/>
+      <c r="D66" s="2" t="inlineStr"/>
+      <c r="E66" s="2" t="inlineStr"/>
+      <c r="F66" s="2" t="inlineStr"/>
+      <c r="G66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="2" t="inlineStr"/>
+      <c r="C67" s="2" t="inlineStr"/>
+      <c r="D67" s="2" t="inlineStr"/>
+      <c r="E67" s="2" t="inlineStr"/>
+      <c r="F67" s="2" t="inlineStr"/>
+      <c r="G67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="2" t="inlineStr"/>
+      <c r="C68" s="2" t="inlineStr"/>
+      <c r="D68" s="2" t="inlineStr"/>
+      <c r="E68" s="2" t="inlineStr"/>
+      <c r="F68" s="2" t="inlineStr"/>
+      <c r="G68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="2" t="inlineStr"/>
+      <c r="C69" s="2" t="inlineStr"/>
+      <c r="D69" s="2" t="inlineStr"/>
+      <c r="E69" s="2" t="inlineStr"/>
+      <c r="F69" s="2" t="inlineStr"/>
+      <c r="G69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" s="2" t="inlineStr"/>
+      <c r="C70" s="2" t="inlineStr"/>
+      <c r="D70" s="2" t="inlineStr"/>
+      <c r="E70" s="2" t="inlineStr"/>
+      <c r="F70" s="2" t="inlineStr"/>
+      <c r="G70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" s="2" t="inlineStr"/>
+      <c r="C71" s="2" t="inlineStr"/>
+      <c r="D71" s="2" t="inlineStr"/>
+      <c r="E71" s="2" t="inlineStr"/>
+      <c r="F71" s="2" t="inlineStr"/>
+      <c r="G71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" s="2" t="inlineStr"/>
+      <c r="C72" s="2" t="inlineStr"/>
+      <c r="D72" s="2" t="inlineStr"/>
+      <c r="E72" s="2" t="inlineStr"/>
+      <c r="F72" s="2" t="inlineStr"/>
+      <c r="G72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" s="2" t="inlineStr"/>
+      <c r="C73" s="2" t="inlineStr"/>
+      <c r="D73" s="2" t="inlineStr"/>
+      <c r="E73" s="2" t="inlineStr"/>
+      <c r="F73" s="2" t="inlineStr"/>
+      <c r="G73" s="2" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" s="2" t="inlineStr"/>
+      <c r="C74" s="2" t="inlineStr"/>
+      <c r="D74" s="2" t="inlineStr"/>
+      <c r="E74" s="2" t="inlineStr"/>
+      <c r="F74" s="2" t="inlineStr"/>
+      <c r="G74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" s="2" t="inlineStr"/>
+      <c r="C75" s="2" t="inlineStr"/>
+      <c r="D75" s="2" t="inlineStr"/>
+      <c r="E75" s="2" t="inlineStr"/>
+      <c r="F75" s="2" t="inlineStr"/>
+      <c r="G75" s="2" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="B76" s="2" t="inlineStr"/>
+      <c r="C76" s="2" t="inlineStr"/>
+      <c r="D76" s="2" t="inlineStr"/>
+      <c r="E76" s="2" t="inlineStr"/>
+      <c r="F76" s="2" t="inlineStr"/>
+      <c r="G76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="n">
+        <v>76</v>
+      </c>
+      <c r="B77" s="2" t="inlineStr"/>
+      <c r="C77" s="2" t="inlineStr"/>
+      <c r="D77" s="2" t="inlineStr"/>
+      <c r="E77" s="2" t="inlineStr"/>
+      <c r="F77" s="2" t="inlineStr"/>
+      <c r="G77" s="2" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="n">
+        <v>77</v>
+      </c>
+      <c r="B78" s="2" t="inlineStr"/>
+      <c r="C78" s="2" t="inlineStr"/>
+      <c r="D78" s="2" t="inlineStr"/>
+      <c r="E78" s="2" t="inlineStr"/>
+      <c r="F78" s="2" t="inlineStr"/>
+      <c r="G78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="B79" s="2" t="inlineStr"/>
+      <c r="C79" s="2" t="inlineStr"/>
+      <c r="D79" s="2" t="inlineStr"/>
+      <c r="E79" s="2" t="inlineStr"/>
+      <c r="F79" s="2" t="inlineStr"/>
+      <c r="G79" s="2" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="n">
+        <v>79</v>
+      </c>
+      <c r="B80" s="2" t="inlineStr"/>
+      <c r="C80" s="2" t="inlineStr"/>
+      <c r="D80" s="2" t="inlineStr"/>
+      <c r="E80" s="2" t="inlineStr"/>
+      <c r="F80" s="2" t="inlineStr"/>
+      <c r="G80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="n">
+        <v>80</v>
+      </c>
+      <c r="B81" s="2" t="inlineStr"/>
+      <c r="C81" s="2" t="inlineStr"/>
+      <c r="D81" s="2" t="inlineStr"/>
+      <c r="E81" s="2" t="inlineStr"/>
+      <c r="F81" s="2" t="inlineStr"/>
+      <c r="G81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="n">
+        <v>81</v>
+      </c>
+      <c r="B82" s="2" t="inlineStr"/>
+      <c r="C82" s="2" t="inlineStr"/>
+      <c r="D82" s="2" t="inlineStr"/>
+      <c r="E82" s="2" t="inlineStr"/>
+      <c r="F82" s="2" t="inlineStr"/>
+      <c r="G82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="B83" s="2" t="inlineStr"/>
+      <c r="C83" s="2" t="inlineStr"/>
+      <c r="D83" s="2" t="inlineStr"/>
+      <c r="E83" s="2" t="inlineStr"/>
+      <c r="F83" s="2" t="inlineStr"/>
+      <c r="G83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="B84" s="2" t="inlineStr"/>
+      <c r="C84" s="2" t="inlineStr"/>
+      <c r="D84" s="2" t="inlineStr"/>
+      <c r="E84" s="2" t="inlineStr"/>
+      <c r="F84" s="2" t="inlineStr"/>
+      <c r="G84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="n">
+        <v>84</v>
+      </c>
+      <c r="B85" s="2" t="inlineStr"/>
+      <c r="C85" s="2" t="inlineStr"/>
+      <c r="D85" s="2" t="inlineStr"/>
+      <c r="E85" s="2" t="inlineStr"/>
+      <c r="F85" s="2" t="inlineStr"/>
+      <c r="G85" s="2" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>85</v>
+      </c>
+      <c r="B86" s="2" t="inlineStr"/>
+      <c r="C86" s="2" t="inlineStr"/>
+      <c r="D86" s="2" t="inlineStr"/>
+      <c r="E86" s="2" t="inlineStr"/>
+      <c r="F86" s="2" t="inlineStr"/>
+      <c r="G86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="B87" s="2" t="inlineStr"/>
+      <c r="C87" s="2" t="inlineStr"/>
+      <c r="D87" s="2" t="inlineStr"/>
+      <c r="E87" s="2" t="inlineStr"/>
+      <c r="F87" s="2" t="inlineStr"/>
+      <c r="G87" s="2" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>87</v>
+      </c>
+      <c r="B88" s="2" t="inlineStr"/>
+      <c r="C88" s="2" t="inlineStr"/>
+      <c r="D88" s="2" t="inlineStr"/>
+      <c r="E88" s="2" t="inlineStr"/>
+      <c r="F88" s="2" t="inlineStr"/>
+      <c r="G88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>88</v>
+      </c>
+      <c r="B89" s="2" t="inlineStr"/>
+      <c r="C89" s="2" t="inlineStr"/>
+      <c r="D89" s="2" t="inlineStr"/>
+      <c r="E89" s="2" t="inlineStr"/>
+      <c r="F89" s="2" t="inlineStr"/>
+      <c r="G89" s="2" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>89</v>
+      </c>
+      <c r="B90" s="2" t="inlineStr"/>
+      <c r="C90" s="2" t="inlineStr"/>
+      <c r="D90" s="2" t="inlineStr"/>
+      <c r="E90" s="2" t="inlineStr"/>
+      <c r="F90" s="2" t="inlineStr"/>
+      <c r="G90" s="2" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>90</v>
+      </c>
+      <c r="B91" s="2" t="inlineStr"/>
+      <c r="C91" s="2" t="inlineStr"/>
+      <c r="D91" s="2" t="inlineStr"/>
+      <c r="E91" s="2" t="inlineStr"/>
+      <c r="F91" s="2" t="inlineStr"/>
+      <c r="G91" s="2" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="n">
+        <v>91</v>
+      </c>
+      <c r="B92" s="2" t="inlineStr"/>
+      <c r="C92" s="2" t="inlineStr"/>
+      <c r="D92" s="2" t="inlineStr"/>
+      <c r="E92" s="2" t="inlineStr"/>
+      <c r="F92" s="2" t="inlineStr"/>
+      <c r="G92" s="2" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="n">
+        <v>92</v>
+      </c>
+      <c r="B93" s="2" t="inlineStr"/>
+      <c r="C93" s="2" t="inlineStr"/>
+      <c r="D93" s="2" t="inlineStr"/>
+      <c r="E93" s="2" t="inlineStr"/>
+      <c r="F93" s="2" t="inlineStr"/>
+      <c r="G93" s="2" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="B94" s="2" t="inlineStr"/>
+      <c r="C94" s="2" t="inlineStr"/>
+      <c r="D94" s="2" t="inlineStr"/>
+      <c r="E94" s="2" t="inlineStr"/>
+      <c r="F94" s="2" t="inlineStr"/>
+      <c r="G94" s="2" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="B95" s="2" t="inlineStr"/>
+      <c r="C95" s="2" t="inlineStr"/>
+      <c r="D95" s="2" t="inlineStr"/>
+      <c r="E95" s="2" t="inlineStr"/>
+      <c r="F95" s="2" t="inlineStr"/>
+      <c r="G95" s="2" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="n">
+        <v>95</v>
+      </c>
+      <c r="B96" s="2" t="inlineStr"/>
+      <c r="C96" s="2" t="inlineStr"/>
+      <c r="D96" s="2" t="inlineStr"/>
+      <c r="E96" s="2" t="inlineStr"/>
+      <c r="F96" s="2" t="inlineStr"/>
+      <c r="G96" s="2" t="inlineStr"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="n">
+        <v>96</v>
+      </c>
+      <c r="B97" s="2" t="inlineStr"/>
+      <c r="C97" s="2" t="inlineStr"/>
+      <c r="D97" s="2" t="inlineStr"/>
+      <c r="E97" s="2" t="inlineStr"/>
+      <c r="F97" s="2" t="inlineStr"/>
+      <c r="G97" s="2" t="inlineStr"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="n">
+        <v>97</v>
+      </c>
+      <c r="B98" s="2" t="inlineStr"/>
+      <c r="C98" s="2" t="inlineStr"/>
+      <c r="D98" s="2" t="inlineStr"/>
+      <c r="E98" s="2" t="inlineStr"/>
+      <c r="F98" s="2" t="inlineStr"/>
+      <c r="G98" s="2" t="inlineStr"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="n">
+        <v>98</v>
+      </c>
+      <c r="B99" s="2" t="inlineStr"/>
+      <c r="C99" s="2" t="inlineStr"/>
+      <c r="D99" s="2" t="inlineStr"/>
+      <c r="E99" s="2" t="inlineStr"/>
+      <c r="F99" s="2" t="inlineStr"/>
+      <c r="G99" s="2" t="inlineStr"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="n">
+        <v>99</v>
+      </c>
+      <c r="B100" s="2" t="inlineStr"/>
+      <c r="C100" s="2" t="inlineStr"/>
+      <c r="D100" s="2" t="inlineStr"/>
+      <c r="E100" s="2" t="inlineStr"/>
+      <c r="F100" s="2" t="inlineStr"/>
+      <c r="G100" s="2" t="inlineStr"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="B101" s="2" t="inlineStr"/>
+      <c r="C101" s="2" t="inlineStr"/>
+      <c r="D101" s="2" t="inlineStr"/>
+      <c r="E101" s="2" t="inlineStr"/>
+      <c r="F101" s="2" t="inlineStr"/>
+      <c r="G101" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:G101"/>
+  <dataValidations count="1">
+    <dataValidation sqref="E2:E101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>'List Dataset'!$B$2:$B$21</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: use star ratings in dataset spreadsheet
</commit_message>
<xml_diff>
--- a/spreadsheet/linear_regression_dataset_spreadsheet.xlsx
+++ b/spreadsheet/linear_regression_dataset_spreadsheet.xlsx
@@ -71,13 +71,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -501,10 +504,12 @@
           <t>Concrete Compressive Strength</t>
         </is>
       </c>
-      <c r="C2" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/165/concrete+compressive+strength</t>
         </is>
@@ -529,10 +534,12 @@
           <t>Energy Efficiency</t>
         </is>
       </c>
-      <c r="C3" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/242/energy+efficiency</t>
         </is>
@@ -557,10 +564,12 @@
           <t>Real Estate Valuation</t>
         </is>
       </c>
-      <c r="C4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/477/real+estate+valuation+data+set</t>
         </is>
@@ -585,10 +594,12 @@
           <t>Auto MPG</t>
         </is>
       </c>
-      <c r="C5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>★★★★</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/9/auto+mpg</t>
         </is>
@@ -613,10 +624,12 @@
           <t>Combined Cycle Power Plant</t>
         </is>
       </c>
-      <c r="C6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/294/combined+cycle+power+plant</t>
         </is>
@@ -641,10 +654,12 @@
           <t>Bike Sharing Dataset</t>
         </is>
       </c>
-      <c r="C7" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/275/bike+sharing+dataset</t>
         </is>
@@ -669,10 +684,12 @@
           <t>Wine Quality</t>
         </is>
       </c>
-      <c r="C8" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>★★</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/186/wine+quality</t>
         </is>
@@ -697,10 +714,12 @@
           <t>Student Performance</t>
         </is>
       </c>
-      <c r="C9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/320/student+performance</t>
         </is>
@@ -725,10 +744,12 @@
           <t>Air Quality</t>
         </is>
       </c>
-      <c r="C10" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/360/air+quality</t>
         </is>
@@ -753,10 +774,12 @@
           <t>Medical Cost Personal Dataset / Insurance</t>
         </is>
       </c>
-      <c r="C11" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D11" s="3" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>★★★★</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
         <is>
           <t>https://www.kaggle.com/datasets/mirichoi0218/insurance</t>
         </is>
@@ -781,10 +804,12 @@
           <t>Fish Market</t>
         </is>
       </c>
-      <c r="C12" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
         <is>
           <t>https://www.kaggle.com/datasets/vipullrathod/fish-market</t>
         </is>
@@ -809,10 +834,12 @@
           <t>Seoul Bike Sharing Demand</t>
         </is>
       </c>
-      <c r="C13" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D13" s="3" t="inlineStr">
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/560/seoul+bike+sharing+demand</t>
         </is>
@@ -837,10 +864,12 @@
           <t>House Rent Prediction Dataset</t>
         </is>
       </c>
-      <c r="C14" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
         <is>
           <t>https://www.kaggle.com/datasets/iamsouravbanerjee/house-rent-prediction-dataset</t>
         </is>
@@ -865,10 +894,12 @@
           <t>Airfoil Self-Noise</t>
         </is>
       </c>
-      <c r="C15" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/291/airfoil+self+noise</t>
         </is>
@@ -893,10 +924,12 @@
           <t>Yacht Hydrodynamics</t>
         </is>
       </c>
-      <c r="C16" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/ml/datasets/yacht+hydrodynamics</t>
         </is>
@@ -921,10 +954,12 @@
           <t>Appliances Energy Prediction</t>
         </is>
       </c>
-      <c r="C17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="D17" s="3" t="inlineStr">
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>★</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/374/appliances+energy+prediction</t>
         </is>
@@ -949,10 +984,12 @@
           <t>Concrete Slump Test</t>
         </is>
       </c>
-      <c r="C18" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>★★★★★</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/182/concrete+slump+test</t>
         </is>
@@ -977,10 +1014,12 @@
           <t>Computer Hardware</t>
         </is>
       </c>
-      <c r="C19" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="D19" s="3" t="inlineStr">
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>★★★★</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/ml/datasets/computer+hardware</t>
         </is>
@@ -1005,10 +1044,12 @@
           <t>QSAR Fish Toxicity</t>
         </is>
       </c>
-      <c r="C20" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/504/qsar+fish+toxicity</t>
         </is>
@@ -1033,10 +1074,12 @@
           <t>Abalone</t>
         </is>
       </c>
-      <c r="C21" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>★★★</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>https://archive.ics.uci.edu/dataset/1/abalone</t>
         </is>
@@ -1099,37 +1142,37 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="4" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="B1" s="4" t="inlineStr">
+      <c r="B1" s="5" t="inlineStr">
         <is>
           <t>Nama</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="5" t="inlineStr">
         <is>
           <t>NIM</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="5" t="inlineStr">
         <is>
           <t>Kelas</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="5" t="inlineStr">
         <is>
           <t>Dataset Yang Diambil</t>
         </is>
       </c>
-      <c r="F1" s="4" t="inlineStr">
+      <c r="F1" s="5" t="inlineStr">
         <is>
           <t>Link Notebook Colab Shared</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Link Pengumpulan Peserta</t>
         </is>

</xml_diff>

<commit_message>
docs: connect submission sheet to dataset list
</commit_message>
<xml_diff>
--- a/spreadsheet/linear_regression_dataset_spreadsheet.xlsx
+++ b/spreadsheet/linear_regression_dataset_spreadsheet.xlsx
@@ -11,8 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pengumpulan" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
+    <definedName name="DatasetList">'List Dataset'!$B$2:$B$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'List Dataset'!$A$1:$F$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pengumpulan'!$A$1:$G$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pengumpulan'!$A$1:$G$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -40,7 +41,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -57,6 +58,11 @@
         <fgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -71,7 +77,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -86,11 +92,26 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="0"/>
   </cellStyles>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="00006100"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00C6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
@@ -1097,6 +1118,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:F21"/>
+  <conditionalFormatting sqref="A2:F21">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>COUNTIFS(Pengumpulan!$E$2:$E$21,$B2,Pengumpulan!$B$2:$B$21,"&lt;&gt;")&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -1129,7 +1155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G101"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1185,7 +1211,7 @@
       <c r="B2" s="2" t="inlineStr"/>
       <c r="C2" s="2" t="inlineStr"/>
       <c r="D2" s="2" t="inlineStr"/>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="6" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
       <c r="G2" s="2" t="inlineStr"/>
     </row>
@@ -1196,7 +1222,7 @@
       <c r="B3" s="2" t="inlineStr"/>
       <c r="C3" s="2" t="inlineStr"/>
       <c r="D3" s="2" t="inlineStr"/>
-      <c r="E3" s="2" t="inlineStr"/>
+      <c r="E3" s="6" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
       <c r="G3" s="2" t="inlineStr"/>
     </row>
@@ -1207,7 +1233,7 @@
       <c r="B4" s="2" t="inlineStr"/>
       <c r="C4" s="2" t="inlineStr"/>
       <c r="D4" s="2" t="inlineStr"/>
-      <c r="E4" s="2" t="inlineStr"/>
+      <c r="E4" s="6" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
       <c r="G4" s="2" t="inlineStr"/>
     </row>
@@ -1218,7 +1244,7 @@
       <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="2" t="inlineStr"/>
       <c r="D5" s="2" t="inlineStr"/>
-      <c r="E5" s="2" t="inlineStr"/>
+      <c r="E5" s="6" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
       <c r="G5" s="2" t="inlineStr"/>
     </row>
@@ -1229,7 +1255,7 @@
       <c r="B6" s="2" t="inlineStr"/>
       <c r="C6" s="2" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr"/>
-      <c r="E6" s="2" t="inlineStr"/>
+      <c r="E6" s="6" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
       <c r="G6" s="2" t="inlineStr"/>
     </row>
@@ -1240,7 +1266,7 @@
       <c r="B7" s="2" t="inlineStr"/>
       <c r="C7" s="2" t="inlineStr"/>
       <c r="D7" s="2" t="inlineStr"/>
-      <c r="E7" s="2" t="inlineStr"/>
+      <c r="E7" s="6" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
       <c r="G7" s="2" t="inlineStr"/>
     </row>
@@ -1251,7 +1277,7 @@
       <c r="B8" s="2" t="inlineStr"/>
       <c r="C8" s="2" t="inlineStr"/>
       <c r="D8" s="2" t="inlineStr"/>
-      <c r="E8" s="2" t="inlineStr"/>
+      <c r="E8" s="6" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
       <c r="G8" s="2" t="inlineStr"/>
     </row>
@@ -1262,7 +1288,7 @@
       <c r="B9" s="2" t="inlineStr"/>
       <c r="C9" s="2" t="inlineStr"/>
       <c r="D9" s="2" t="inlineStr"/>
-      <c r="E9" s="2" t="inlineStr"/>
+      <c r="E9" s="6" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr"/>
       <c r="G9" s="2" t="inlineStr"/>
     </row>
@@ -1273,7 +1299,7 @@
       <c r="B10" s="2" t="inlineStr"/>
       <c r="C10" s="2" t="inlineStr"/>
       <c r="D10" s="2" t="inlineStr"/>
-      <c r="E10" s="2" t="inlineStr"/>
+      <c r="E10" s="6" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
       <c r="G10" s="2" t="inlineStr"/>
     </row>
@@ -1284,7 +1310,7 @@
       <c r="B11" s="2" t="inlineStr"/>
       <c r="C11" s="2" t="inlineStr"/>
       <c r="D11" s="2" t="inlineStr"/>
-      <c r="E11" s="2" t="inlineStr"/>
+      <c r="E11" s="6" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
       <c r="G11" s="2" t="inlineStr"/>
     </row>
@@ -1295,7 +1321,7 @@
       <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="2" t="inlineStr"/>
       <c r="D12" s="2" t="inlineStr"/>
-      <c r="E12" s="2" t="inlineStr"/>
+      <c r="E12" s="6" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
       <c r="G12" s="2" t="inlineStr"/>
     </row>
@@ -1306,7 +1332,7 @@
       <c r="B13" s="2" t="inlineStr"/>
       <c r="C13" s="2" t="inlineStr"/>
       <c r="D13" s="2" t="inlineStr"/>
-      <c r="E13" s="2" t="inlineStr"/>
+      <c r="E13" s="6" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
       <c r="G13" s="2" t="inlineStr"/>
     </row>
@@ -1317,7 +1343,7 @@
       <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="2" t="inlineStr"/>
       <c r="D14" s="2" t="inlineStr"/>
-      <c r="E14" s="2" t="inlineStr"/>
+      <c r="E14" s="6" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
       <c r="G14" s="2" t="inlineStr"/>
     </row>
@@ -1328,7 +1354,7 @@
       <c r="B15" s="2" t="inlineStr"/>
       <c r="C15" s="2" t="inlineStr"/>
       <c r="D15" s="2" t="inlineStr"/>
-      <c r="E15" s="2" t="inlineStr"/>
+      <c r="E15" s="6" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
       <c r="G15" s="2" t="inlineStr"/>
     </row>
@@ -1339,7 +1365,7 @@
       <c r="B16" s="2" t="inlineStr"/>
       <c r="C16" s="2" t="inlineStr"/>
       <c r="D16" s="2" t="inlineStr"/>
-      <c r="E16" s="2" t="inlineStr"/>
+      <c r="E16" s="6" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
       <c r="G16" s="2" t="inlineStr"/>
     </row>
@@ -1350,7 +1376,7 @@
       <c r="B17" s="2" t="inlineStr"/>
       <c r="C17" s="2" t="inlineStr"/>
       <c r="D17" s="2" t="inlineStr"/>
-      <c r="E17" s="2" t="inlineStr"/>
+      <c r="E17" s="6" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
       <c r="G17" s="2" t="inlineStr"/>
     </row>
@@ -1361,7 +1387,7 @@
       <c r="B18" s="2" t="inlineStr"/>
       <c r="C18" s="2" t="inlineStr"/>
       <c r="D18" s="2" t="inlineStr"/>
-      <c r="E18" s="2" t="inlineStr"/>
+      <c r="E18" s="6" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
       <c r="G18" s="2" t="inlineStr"/>
     </row>
@@ -1372,7 +1398,7 @@
       <c r="B19" s="2" t="inlineStr"/>
       <c r="C19" s="2" t="inlineStr"/>
       <c r="D19" s="2" t="inlineStr"/>
-      <c r="E19" s="2" t="inlineStr"/>
+      <c r="E19" s="6" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
       <c r="G19" s="2" t="inlineStr"/>
     </row>
@@ -1383,7 +1409,7 @@
       <c r="B20" s="2" t="inlineStr"/>
       <c r="C20" s="2" t="inlineStr"/>
       <c r="D20" s="2" t="inlineStr"/>
-      <c r="E20" s="2" t="inlineStr"/>
+      <c r="E20" s="6" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
       <c r="G20" s="2" t="inlineStr"/>
     </row>
@@ -1394,895 +1420,15 @@
       <c r="B21" s="2" t="inlineStr"/>
       <c r="C21" s="2" t="inlineStr"/>
       <c r="D21" s="2" t="inlineStr"/>
-      <c r="E21" s="2" t="inlineStr"/>
+      <c r="E21" s="6" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
       <c r="G21" s="2" t="inlineStr"/>
     </row>
-    <row r="22">
-      <c r="A22" s="2" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" s="2" t="inlineStr"/>
-      <c r="C22" s="2" t="inlineStr"/>
-      <c r="D22" s="2" t="inlineStr"/>
-      <c r="E22" s="2" t="inlineStr"/>
-      <c r="F22" s="2" t="inlineStr"/>
-      <c r="G22" s="2" t="inlineStr"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" s="2" t="inlineStr"/>
-      <c r="C23" s="2" t="inlineStr"/>
-      <c r="D23" s="2" t="inlineStr"/>
-      <c r="E23" s="2" t="inlineStr"/>
-      <c r="F23" s="2" t="inlineStr"/>
-      <c r="G23" s="2" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" s="2" t="inlineStr"/>
-      <c r="C24" s="2" t="inlineStr"/>
-      <c r="D24" s="2" t="inlineStr"/>
-      <c r="E24" s="2" t="inlineStr"/>
-      <c r="F24" s="2" t="inlineStr"/>
-      <c r="G24" s="2" t="inlineStr"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" s="2" t="inlineStr"/>
-      <c r="C25" s="2" t="inlineStr"/>
-      <c r="D25" s="2" t="inlineStr"/>
-      <c r="E25" s="2" t="inlineStr"/>
-      <c r="F25" s="2" t="inlineStr"/>
-      <c r="G25" s="2" t="inlineStr"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" s="2" t="inlineStr"/>
-      <c r="C26" s="2" t="inlineStr"/>
-      <c r="D26" s="2" t="inlineStr"/>
-      <c r="E26" s="2" t="inlineStr"/>
-      <c r="F26" s="2" t="inlineStr"/>
-      <c r="G26" s="2" t="inlineStr"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="2" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" s="2" t="inlineStr"/>
-      <c r="C27" s="2" t="inlineStr"/>
-      <c r="D27" s="2" t="inlineStr"/>
-      <c r="E27" s="2" t="inlineStr"/>
-      <c r="F27" s="2" t="inlineStr"/>
-      <c r="G27" s="2" t="inlineStr"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="2" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" s="2" t="inlineStr"/>
-      <c r="C28" s="2" t="inlineStr"/>
-      <c r="D28" s="2" t="inlineStr"/>
-      <c r="E28" s="2" t="inlineStr"/>
-      <c r="F28" s="2" t="inlineStr"/>
-      <c r="G28" s="2" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="2" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" s="2" t="inlineStr"/>
-      <c r="C29" s="2" t="inlineStr"/>
-      <c r="D29" s="2" t="inlineStr"/>
-      <c r="E29" s="2" t="inlineStr"/>
-      <c r="F29" s="2" t="inlineStr"/>
-      <c r="G29" s="2" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="2" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" s="2" t="inlineStr"/>
-      <c r="C30" s="2" t="inlineStr"/>
-      <c r="D30" s="2" t="inlineStr"/>
-      <c r="E30" s="2" t="inlineStr"/>
-      <c r="F30" s="2" t="inlineStr"/>
-      <c r="G30" s="2" t="inlineStr"/>
-    </row>
-    <row r="31">
-      <c r="A31" s="2" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" s="2" t="inlineStr"/>
-      <c r="C31" s="2" t="inlineStr"/>
-      <c r="D31" s="2" t="inlineStr"/>
-      <c r="E31" s="2" t="inlineStr"/>
-      <c r="F31" s="2" t="inlineStr"/>
-      <c r="G31" s="2" t="inlineStr"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="2" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" s="2" t="inlineStr"/>
-      <c r="C32" s="2" t="inlineStr"/>
-      <c r="D32" s="2" t="inlineStr"/>
-      <c r="E32" s="2" t="inlineStr"/>
-      <c r="F32" s="2" t="inlineStr"/>
-      <c r="G32" s="2" t="inlineStr"/>
-    </row>
-    <row r="33">
-      <c r="A33" s="2" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" s="2" t="inlineStr"/>
-      <c r="C33" s="2" t="inlineStr"/>
-      <c r="D33" s="2" t="inlineStr"/>
-      <c r="E33" s="2" t="inlineStr"/>
-      <c r="F33" s="2" t="inlineStr"/>
-      <c r="G33" s="2" t="inlineStr"/>
-    </row>
-    <row r="34">
-      <c r="A34" s="2" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" s="2" t="inlineStr"/>
-      <c r="C34" s="2" t="inlineStr"/>
-      <c r="D34" s="2" t="inlineStr"/>
-      <c r="E34" s="2" t="inlineStr"/>
-      <c r="F34" s="2" t="inlineStr"/>
-      <c r="G34" s="2" t="inlineStr"/>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" s="2" t="inlineStr"/>
-      <c r="C35" s="2" t="inlineStr"/>
-      <c r="D35" s="2" t="inlineStr"/>
-      <c r="E35" s="2" t="inlineStr"/>
-      <c r="F35" s="2" t="inlineStr"/>
-      <c r="G35" s="2" t="inlineStr"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="2" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" s="2" t="inlineStr"/>
-      <c r="C36" s="2" t="inlineStr"/>
-      <c r="D36" s="2" t="inlineStr"/>
-      <c r="E36" s="2" t="inlineStr"/>
-      <c r="F36" s="2" t="inlineStr"/>
-      <c r="G36" s="2" t="inlineStr"/>
-    </row>
-    <row r="37">
-      <c r="A37" s="2" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" s="2" t="inlineStr"/>
-      <c r="C37" s="2" t="inlineStr"/>
-      <c r="D37" s="2" t="inlineStr"/>
-      <c r="E37" s="2" t="inlineStr"/>
-      <c r="F37" s="2" t="inlineStr"/>
-      <c r="G37" s="2" t="inlineStr"/>
-    </row>
-    <row r="38">
-      <c r="A38" s="2" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" s="2" t="inlineStr"/>
-      <c r="C38" s="2" t="inlineStr"/>
-      <c r="D38" s="2" t="inlineStr"/>
-      <c r="E38" s="2" t="inlineStr"/>
-      <c r="F38" s="2" t="inlineStr"/>
-      <c r="G38" s="2" t="inlineStr"/>
-    </row>
-    <row r="39">
-      <c r="A39" s="2" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" s="2" t="inlineStr"/>
-      <c r="C39" s="2" t="inlineStr"/>
-      <c r="D39" s="2" t="inlineStr"/>
-      <c r="E39" s="2" t="inlineStr"/>
-      <c r="F39" s="2" t="inlineStr"/>
-      <c r="G39" s="2" t="inlineStr"/>
-    </row>
-    <row r="40">
-      <c r="A40" s="2" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" s="2" t="inlineStr"/>
-      <c r="C40" s="2" t="inlineStr"/>
-      <c r="D40" s="2" t="inlineStr"/>
-      <c r="E40" s="2" t="inlineStr"/>
-      <c r="F40" s="2" t="inlineStr"/>
-      <c r="G40" s="2" t="inlineStr"/>
-    </row>
-    <row r="41">
-      <c r="A41" s="2" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" s="2" t="inlineStr"/>
-      <c r="C41" s="2" t="inlineStr"/>
-      <c r="D41" s="2" t="inlineStr"/>
-      <c r="E41" s="2" t="inlineStr"/>
-      <c r="F41" s="2" t="inlineStr"/>
-      <c r="G41" s="2" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" s="2" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" s="2" t="inlineStr"/>
-      <c r="C42" s="2" t="inlineStr"/>
-      <c r="D42" s="2" t="inlineStr"/>
-      <c r="E42" s="2" t="inlineStr"/>
-      <c r="F42" s="2" t="inlineStr"/>
-      <c r="G42" s="2" t="inlineStr"/>
-    </row>
-    <row r="43">
-      <c r="A43" s="2" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" s="2" t="inlineStr"/>
-      <c r="C43" s="2" t="inlineStr"/>
-      <c r="D43" s="2" t="inlineStr"/>
-      <c r="E43" s="2" t="inlineStr"/>
-      <c r="F43" s="2" t="inlineStr"/>
-      <c r="G43" s="2" t="inlineStr"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="2" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" s="2" t="inlineStr"/>
-      <c r="C44" s="2" t="inlineStr"/>
-      <c r="D44" s="2" t="inlineStr"/>
-      <c r="E44" s="2" t="inlineStr"/>
-      <c r="F44" s="2" t="inlineStr"/>
-      <c r="G44" s="2" t="inlineStr"/>
-    </row>
-    <row r="45">
-      <c r="A45" s="2" t="n">
-        <v>44</v>
-      </c>
-      <c r="B45" s="2" t="inlineStr"/>
-      <c r="C45" s="2" t="inlineStr"/>
-      <c r="D45" s="2" t="inlineStr"/>
-      <c r="E45" s="2" t="inlineStr"/>
-      <c r="F45" s="2" t="inlineStr"/>
-      <c r="G45" s="2" t="inlineStr"/>
-    </row>
-    <row r="46">
-      <c r="A46" s="2" t="n">
-        <v>45</v>
-      </c>
-      <c r="B46" s="2" t="inlineStr"/>
-      <c r="C46" s="2" t="inlineStr"/>
-      <c r="D46" s="2" t="inlineStr"/>
-      <c r="E46" s="2" t="inlineStr"/>
-      <c r="F46" s="2" t="inlineStr"/>
-      <c r="G46" s="2" t="inlineStr"/>
-    </row>
-    <row r="47">
-      <c r="A47" s="2" t="n">
-        <v>46</v>
-      </c>
-      <c r="B47" s="2" t="inlineStr"/>
-      <c r="C47" s="2" t="inlineStr"/>
-      <c r="D47" s="2" t="inlineStr"/>
-      <c r="E47" s="2" t="inlineStr"/>
-      <c r="F47" s="2" t="inlineStr"/>
-      <c r="G47" s="2" t="inlineStr"/>
-    </row>
-    <row r="48">
-      <c r="A48" s="2" t="n">
-        <v>47</v>
-      </c>
-      <c r="B48" s="2" t="inlineStr"/>
-      <c r="C48" s="2" t="inlineStr"/>
-      <c r="D48" s="2" t="inlineStr"/>
-      <c r="E48" s="2" t="inlineStr"/>
-      <c r="F48" s="2" t="inlineStr"/>
-      <c r="G48" s="2" t="inlineStr"/>
-    </row>
-    <row r="49">
-      <c r="A49" s="2" t="n">
-        <v>48</v>
-      </c>
-      <c r="B49" s="2" t="inlineStr"/>
-      <c r="C49" s="2" t="inlineStr"/>
-      <c r="D49" s="2" t="inlineStr"/>
-      <c r="E49" s="2" t="inlineStr"/>
-      <c r="F49" s="2" t="inlineStr"/>
-      <c r="G49" s="2" t="inlineStr"/>
-    </row>
-    <row r="50">
-      <c r="A50" s="2" t="n">
-        <v>49</v>
-      </c>
-      <c r="B50" s="2" t="inlineStr"/>
-      <c r="C50" s="2" t="inlineStr"/>
-      <c r="D50" s="2" t="inlineStr"/>
-      <c r="E50" s="2" t="inlineStr"/>
-      <c r="F50" s="2" t="inlineStr"/>
-      <c r="G50" s="2" t="inlineStr"/>
-    </row>
-    <row r="51">
-      <c r="A51" s="2" t="n">
-        <v>50</v>
-      </c>
-      <c r="B51" s="2" t="inlineStr"/>
-      <c r="C51" s="2" t="inlineStr"/>
-      <c r="D51" s="2" t="inlineStr"/>
-      <c r="E51" s="2" t="inlineStr"/>
-      <c r="F51" s="2" t="inlineStr"/>
-      <c r="G51" s="2" t="inlineStr"/>
-    </row>
-    <row r="52">
-      <c r="A52" s="2" t="n">
-        <v>51</v>
-      </c>
-      <c r="B52" s="2" t="inlineStr"/>
-      <c r="C52" s="2" t="inlineStr"/>
-      <c r="D52" s="2" t="inlineStr"/>
-      <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="2" t="inlineStr"/>
-      <c r="G52" s="2" t="inlineStr"/>
-    </row>
-    <row r="53">
-      <c r="A53" s="2" t="n">
-        <v>52</v>
-      </c>
-      <c r="B53" s="2" t="inlineStr"/>
-      <c r="C53" s="2" t="inlineStr"/>
-      <c r="D53" s="2" t="inlineStr"/>
-      <c r="E53" s="2" t="inlineStr"/>
-      <c r="F53" s="2" t="inlineStr"/>
-      <c r="G53" s="2" t="inlineStr"/>
-    </row>
-    <row r="54">
-      <c r="A54" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="B54" s="2" t="inlineStr"/>
-      <c r="C54" s="2" t="inlineStr"/>
-      <c r="D54" s="2" t="inlineStr"/>
-      <c r="E54" s="2" t="inlineStr"/>
-      <c r="F54" s="2" t="inlineStr"/>
-      <c r="G54" s="2" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="B55" s="2" t="inlineStr"/>
-      <c r="C55" s="2" t="inlineStr"/>
-      <c r="D55" s="2" t="inlineStr"/>
-      <c r="E55" s="2" t="inlineStr"/>
-      <c r="F55" s="2" t="inlineStr"/>
-      <c r="G55" s="2" t="inlineStr"/>
-    </row>
-    <row r="56">
-      <c r="A56" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="B56" s="2" t="inlineStr"/>
-      <c r="C56" s="2" t="inlineStr"/>
-      <c r="D56" s="2" t="inlineStr"/>
-      <c r="E56" s="2" t="inlineStr"/>
-      <c r="F56" s="2" t="inlineStr"/>
-      <c r="G56" s="2" t="inlineStr"/>
-    </row>
-    <row r="57">
-      <c r="A57" s="2" t="n">
-        <v>56</v>
-      </c>
-      <c r="B57" s="2" t="inlineStr"/>
-      <c r="C57" s="2" t="inlineStr"/>
-      <c r="D57" s="2" t="inlineStr"/>
-      <c r="E57" s="2" t="inlineStr"/>
-      <c r="F57" s="2" t="inlineStr"/>
-      <c r="G57" s="2" t="inlineStr"/>
-    </row>
-    <row r="58">
-      <c r="A58" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="B58" s="2" t="inlineStr"/>
-      <c r="C58" s="2" t="inlineStr"/>
-      <c r="D58" s="2" t="inlineStr"/>
-      <c r="E58" s="2" t="inlineStr"/>
-      <c r="F58" s="2" t="inlineStr"/>
-      <c r="G58" s="2" t="inlineStr"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="B59" s="2" t="inlineStr"/>
-      <c r="C59" s="2" t="inlineStr"/>
-      <c r="D59" s="2" t="inlineStr"/>
-      <c r="E59" s="2" t="inlineStr"/>
-      <c r="F59" s="2" t="inlineStr"/>
-      <c r="G59" s="2" t="inlineStr"/>
-    </row>
-    <row r="60">
-      <c r="A60" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="B60" s="2" t="inlineStr"/>
-      <c r="C60" s="2" t="inlineStr"/>
-      <c r="D60" s="2" t="inlineStr"/>
-      <c r="E60" s="2" t="inlineStr"/>
-      <c r="F60" s="2" t="inlineStr"/>
-      <c r="G60" s="2" t="inlineStr"/>
-    </row>
-    <row r="61">
-      <c r="A61" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="B61" s="2" t="inlineStr"/>
-      <c r="C61" s="2" t="inlineStr"/>
-      <c r="D61" s="2" t="inlineStr"/>
-      <c r="E61" s="2" t="inlineStr"/>
-      <c r="F61" s="2" t="inlineStr"/>
-      <c r="G61" s="2" t="inlineStr"/>
-    </row>
-    <row r="62">
-      <c r="A62" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="B62" s="2" t="inlineStr"/>
-      <c r="C62" s="2" t="inlineStr"/>
-      <c r="D62" s="2" t="inlineStr"/>
-      <c r="E62" s="2" t="inlineStr"/>
-      <c r="F62" s="2" t="inlineStr"/>
-      <c r="G62" s="2" t="inlineStr"/>
-    </row>
-    <row r="63">
-      <c r="A63" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="B63" s="2" t="inlineStr"/>
-      <c r="C63" s="2" t="inlineStr"/>
-      <c r="D63" s="2" t="inlineStr"/>
-      <c r="E63" s="2" t="inlineStr"/>
-      <c r="F63" s="2" t="inlineStr"/>
-      <c r="G63" s="2" t="inlineStr"/>
-    </row>
-    <row r="64">
-      <c r="A64" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="B64" s="2" t="inlineStr"/>
-      <c r="C64" s="2" t="inlineStr"/>
-      <c r="D64" s="2" t="inlineStr"/>
-      <c r="E64" s="2" t="inlineStr"/>
-      <c r="F64" s="2" t="inlineStr"/>
-      <c r="G64" s="2" t="inlineStr"/>
-    </row>
-    <row r="65">
-      <c r="A65" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="B65" s="2" t="inlineStr"/>
-      <c r="C65" s="2" t="inlineStr"/>
-      <c r="D65" s="2" t="inlineStr"/>
-      <c r="E65" s="2" t="inlineStr"/>
-      <c r="F65" s="2" t="inlineStr"/>
-      <c r="G65" s="2" t="inlineStr"/>
-    </row>
-    <row r="66">
-      <c r="A66" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="B66" s="2" t="inlineStr"/>
-      <c r="C66" s="2" t="inlineStr"/>
-      <c r="D66" s="2" t="inlineStr"/>
-      <c r="E66" s="2" t="inlineStr"/>
-      <c r="F66" s="2" t="inlineStr"/>
-      <c r="G66" s="2" t="inlineStr"/>
-    </row>
-    <row r="67">
-      <c r="A67" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="B67" s="2" t="inlineStr"/>
-      <c r="C67" s="2" t="inlineStr"/>
-      <c r="D67" s="2" t="inlineStr"/>
-      <c r="E67" s="2" t="inlineStr"/>
-      <c r="F67" s="2" t="inlineStr"/>
-      <c r="G67" s="2" t="inlineStr"/>
-    </row>
-    <row r="68">
-      <c r="A68" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="B68" s="2" t="inlineStr"/>
-      <c r="C68" s="2" t="inlineStr"/>
-      <c r="D68" s="2" t="inlineStr"/>
-      <c r="E68" s="2" t="inlineStr"/>
-      <c r="F68" s="2" t="inlineStr"/>
-      <c r="G68" s="2" t="inlineStr"/>
-    </row>
-    <row r="69">
-      <c r="A69" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="B69" s="2" t="inlineStr"/>
-      <c r="C69" s="2" t="inlineStr"/>
-      <c r="D69" s="2" t="inlineStr"/>
-      <c r="E69" s="2" t="inlineStr"/>
-      <c r="F69" s="2" t="inlineStr"/>
-      <c r="G69" s="2" t="inlineStr"/>
-    </row>
-    <row r="70">
-      <c r="A70" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="B70" s="2" t="inlineStr"/>
-      <c r="C70" s="2" t="inlineStr"/>
-      <c r="D70" s="2" t="inlineStr"/>
-      <c r="E70" s="2" t="inlineStr"/>
-      <c r="F70" s="2" t="inlineStr"/>
-      <c r="G70" s="2" t="inlineStr"/>
-    </row>
-    <row r="71">
-      <c r="A71" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="B71" s="2" t="inlineStr"/>
-      <c r="C71" s="2" t="inlineStr"/>
-      <c r="D71" s="2" t="inlineStr"/>
-      <c r="E71" s="2" t="inlineStr"/>
-      <c r="F71" s="2" t="inlineStr"/>
-      <c r="G71" s="2" t="inlineStr"/>
-    </row>
-    <row r="72">
-      <c r="A72" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="B72" s="2" t="inlineStr"/>
-      <c r="C72" s="2" t="inlineStr"/>
-      <c r="D72" s="2" t="inlineStr"/>
-      <c r="E72" s="2" t="inlineStr"/>
-      <c r="F72" s="2" t="inlineStr"/>
-      <c r="G72" s="2" t="inlineStr"/>
-    </row>
-    <row r="73">
-      <c r="A73" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="B73" s="2" t="inlineStr"/>
-      <c r="C73" s="2" t="inlineStr"/>
-      <c r="D73" s="2" t="inlineStr"/>
-      <c r="E73" s="2" t="inlineStr"/>
-      <c r="F73" s="2" t="inlineStr"/>
-      <c r="G73" s="2" t="inlineStr"/>
-    </row>
-    <row r="74">
-      <c r="A74" s="2" t="n">
-        <v>73</v>
-      </c>
-      <c r="B74" s="2" t="inlineStr"/>
-      <c r="C74" s="2" t="inlineStr"/>
-      <c r="D74" s="2" t="inlineStr"/>
-      <c r="E74" s="2" t="inlineStr"/>
-      <c r="F74" s="2" t="inlineStr"/>
-      <c r="G74" s="2" t="inlineStr"/>
-    </row>
-    <row r="75">
-      <c r="A75" s="2" t="n">
-        <v>74</v>
-      </c>
-      <c r="B75" s="2" t="inlineStr"/>
-      <c r="C75" s="2" t="inlineStr"/>
-      <c r="D75" s="2" t="inlineStr"/>
-      <c r="E75" s="2" t="inlineStr"/>
-      <c r="F75" s="2" t="inlineStr"/>
-      <c r="G75" s="2" t="inlineStr"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="B76" s="2" t="inlineStr"/>
-      <c r="C76" s="2" t="inlineStr"/>
-      <c r="D76" s="2" t="inlineStr"/>
-      <c r="E76" s="2" t="inlineStr"/>
-      <c r="F76" s="2" t="inlineStr"/>
-      <c r="G76" s="2" t="inlineStr"/>
-    </row>
-    <row r="77">
-      <c r="A77" s="2" t="n">
-        <v>76</v>
-      </c>
-      <c r="B77" s="2" t="inlineStr"/>
-      <c r="C77" s="2" t="inlineStr"/>
-      <c r="D77" s="2" t="inlineStr"/>
-      <c r="E77" s="2" t="inlineStr"/>
-      <c r="F77" s="2" t="inlineStr"/>
-      <c r="G77" s="2" t="inlineStr"/>
-    </row>
-    <row r="78">
-      <c r="A78" s="2" t="n">
-        <v>77</v>
-      </c>
-      <c r="B78" s="2" t="inlineStr"/>
-      <c r="C78" s="2" t="inlineStr"/>
-      <c r="D78" s="2" t="inlineStr"/>
-      <c r="E78" s="2" t="inlineStr"/>
-      <c r="F78" s="2" t="inlineStr"/>
-      <c r="G78" s="2" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="B79" s="2" t="inlineStr"/>
-      <c r="C79" s="2" t="inlineStr"/>
-      <c r="D79" s="2" t="inlineStr"/>
-      <c r="E79" s="2" t="inlineStr"/>
-      <c r="F79" s="2" t="inlineStr"/>
-      <c r="G79" s="2" t="inlineStr"/>
-    </row>
-    <row r="80">
-      <c r="A80" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="B80" s="2" t="inlineStr"/>
-      <c r="C80" s="2" t="inlineStr"/>
-      <c r="D80" s="2" t="inlineStr"/>
-      <c r="E80" s="2" t="inlineStr"/>
-      <c r="F80" s="2" t="inlineStr"/>
-      <c r="G80" s="2" t="inlineStr"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="B81" s="2" t="inlineStr"/>
-      <c r="C81" s="2" t="inlineStr"/>
-      <c r="D81" s="2" t="inlineStr"/>
-      <c r="E81" s="2" t="inlineStr"/>
-      <c r="F81" s="2" t="inlineStr"/>
-      <c r="G81" s="2" t="inlineStr"/>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="n">
-        <v>81</v>
-      </c>
-      <c r="B82" s="2" t="inlineStr"/>
-      <c r="C82" s="2" t="inlineStr"/>
-      <c r="D82" s="2" t="inlineStr"/>
-      <c r="E82" s="2" t="inlineStr"/>
-      <c r="F82" s="2" t="inlineStr"/>
-      <c r="G82" s="2" t="inlineStr"/>
-    </row>
-    <row r="83">
-      <c r="A83" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="B83" s="2" t="inlineStr"/>
-      <c r="C83" s="2" t="inlineStr"/>
-      <c r="D83" s="2" t="inlineStr"/>
-      <c r="E83" s="2" t="inlineStr"/>
-      <c r="F83" s="2" t="inlineStr"/>
-      <c r="G83" s="2" t="inlineStr"/>
-    </row>
-    <row r="84">
-      <c r="A84" s="2" t="n">
-        <v>83</v>
-      </c>
-      <c r="B84" s="2" t="inlineStr"/>
-      <c r="C84" s="2" t="inlineStr"/>
-      <c r="D84" s="2" t="inlineStr"/>
-      <c r="E84" s="2" t="inlineStr"/>
-      <c r="F84" s="2" t="inlineStr"/>
-      <c r="G84" s="2" t="inlineStr"/>
-    </row>
-    <row r="85">
-      <c r="A85" s="2" t="n">
-        <v>84</v>
-      </c>
-      <c r="B85" s="2" t="inlineStr"/>
-      <c r="C85" s="2" t="inlineStr"/>
-      <c r="D85" s="2" t="inlineStr"/>
-      <c r="E85" s="2" t="inlineStr"/>
-      <c r="F85" s="2" t="inlineStr"/>
-      <c r="G85" s="2" t="inlineStr"/>
-    </row>
-    <row r="86">
-      <c r="A86" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="B86" s="2" t="inlineStr"/>
-      <c r="C86" s="2" t="inlineStr"/>
-      <c r="D86" s="2" t="inlineStr"/>
-      <c r="E86" s="2" t="inlineStr"/>
-      <c r="F86" s="2" t="inlineStr"/>
-      <c r="G86" s="2" t="inlineStr"/>
-    </row>
-    <row r="87">
-      <c r="A87" s="2" t="n">
-        <v>86</v>
-      </c>
-      <c r="B87" s="2" t="inlineStr"/>
-      <c r="C87" s="2" t="inlineStr"/>
-      <c r="D87" s="2" t="inlineStr"/>
-      <c r="E87" s="2" t="inlineStr"/>
-      <c r="F87" s="2" t="inlineStr"/>
-      <c r="G87" s="2" t="inlineStr"/>
-    </row>
-    <row r="88">
-      <c r="A88" s="2" t="n">
-        <v>87</v>
-      </c>
-      <c r="B88" s="2" t="inlineStr"/>
-      <c r="C88" s="2" t="inlineStr"/>
-      <c r="D88" s="2" t="inlineStr"/>
-      <c r="E88" s="2" t="inlineStr"/>
-      <c r="F88" s="2" t="inlineStr"/>
-      <c r="G88" s="2" t="inlineStr"/>
-    </row>
-    <row r="89">
-      <c r="A89" s="2" t="n">
-        <v>88</v>
-      </c>
-      <c r="B89" s="2" t="inlineStr"/>
-      <c r="C89" s="2" t="inlineStr"/>
-      <c r="D89" s="2" t="inlineStr"/>
-      <c r="E89" s="2" t="inlineStr"/>
-      <c r="F89" s="2" t="inlineStr"/>
-      <c r="G89" s="2" t="inlineStr"/>
-    </row>
-    <row r="90">
-      <c r="A90" s="2" t="n">
-        <v>89</v>
-      </c>
-      <c r="B90" s="2" t="inlineStr"/>
-      <c r="C90" s="2" t="inlineStr"/>
-      <c r="D90" s="2" t="inlineStr"/>
-      <c r="E90" s="2" t="inlineStr"/>
-      <c r="F90" s="2" t="inlineStr"/>
-      <c r="G90" s="2" t="inlineStr"/>
-    </row>
-    <row r="91">
-      <c r="A91" s="2" t="n">
-        <v>90</v>
-      </c>
-      <c r="B91" s="2" t="inlineStr"/>
-      <c r="C91" s="2" t="inlineStr"/>
-      <c r="D91" s="2" t="inlineStr"/>
-      <c r="E91" s="2" t="inlineStr"/>
-      <c r="F91" s="2" t="inlineStr"/>
-      <c r="G91" s="2" t="inlineStr"/>
-    </row>
-    <row r="92">
-      <c r="A92" s="2" t="n">
-        <v>91</v>
-      </c>
-      <c r="B92" s="2" t="inlineStr"/>
-      <c r="C92" s="2" t="inlineStr"/>
-      <c r="D92" s="2" t="inlineStr"/>
-      <c r="E92" s="2" t="inlineStr"/>
-      <c r="F92" s="2" t="inlineStr"/>
-      <c r="G92" s="2" t="inlineStr"/>
-    </row>
-    <row r="93">
-      <c r="A93" s="2" t="n">
-        <v>92</v>
-      </c>
-      <c r="B93" s="2" t="inlineStr"/>
-      <c r="C93" s="2" t="inlineStr"/>
-      <c r="D93" s="2" t="inlineStr"/>
-      <c r="E93" s="2" t="inlineStr"/>
-      <c r="F93" s="2" t="inlineStr"/>
-      <c r="G93" s="2" t="inlineStr"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="2" t="n">
-        <v>93</v>
-      </c>
-      <c r="B94" s="2" t="inlineStr"/>
-      <c r="C94" s="2" t="inlineStr"/>
-      <c r="D94" s="2" t="inlineStr"/>
-      <c r="E94" s="2" t="inlineStr"/>
-      <c r="F94" s="2" t="inlineStr"/>
-      <c r="G94" s="2" t="inlineStr"/>
-    </row>
-    <row r="95">
-      <c r="A95" s="2" t="n">
-        <v>94</v>
-      </c>
-      <c r="B95" s="2" t="inlineStr"/>
-      <c r="C95" s="2" t="inlineStr"/>
-      <c r="D95" s="2" t="inlineStr"/>
-      <c r="E95" s="2" t="inlineStr"/>
-      <c r="F95" s="2" t="inlineStr"/>
-      <c r="G95" s="2" t="inlineStr"/>
-    </row>
-    <row r="96">
-      <c r="A96" s="2" t="n">
-        <v>95</v>
-      </c>
-      <c r="B96" s="2" t="inlineStr"/>
-      <c r="C96" s="2" t="inlineStr"/>
-      <c r="D96" s="2" t="inlineStr"/>
-      <c r="E96" s="2" t="inlineStr"/>
-      <c r="F96" s="2" t="inlineStr"/>
-      <c r="G96" s="2" t="inlineStr"/>
-    </row>
-    <row r="97">
-      <c r="A97" s="2" t="n">
-        <v>96</v>
-      </c>
-      <c r="B97" s="2" t="inlineStr"/>
-      <c r="C97" s="2" t="inlineStr"/>
-      <c r="D97" s="2" t="inlineStr"/>
-      <c r="E97" s="2" t="inlineStr"/>
-      <c r="F97" s="2" t="inlineStr"/>
-      <c r="G97" s="2" t="inlineStr"/>
-    </row>
-    <row r="98">
-      <c r="A98" s="2" t="n">
-        <v>97</v>
-      </c>
-      <c r="B98" s="2" t="inlineStr"/>
-      <c r="C98" s="2" t="inlineStr"/>
-      <c r="D98" s="2" t="inlineStr"/>
-      <c r="E98" s="2" t="inlineStr"/>
-      <c r="F98" s="2" t="inlineStr"/>
-      <c r="G98" s="2" t="inlineStr"/>
-    </row>
-    <row r="99">
-      <c r="A99" s="2" t="n">
-        <v>98</v>
-      </c>
-      <c r="B99" s="2" t="inlineStr"/>
-      <c r="C99" s="2" t="inlineStr"/>
-      <c r="D99" s="2" t="inlineStr"/>
-      <c r="E99" s="2" t="inlineStr"/>
-      <c r="F99" s="2" t="inlineStr"/>
-      <c r="G99" s="2" t="inlineStr"/>
-    </row>
-    <row r="100">
-      <c r="A100" s="2" t="n">
-        <v>99</v>
-      </c>
-      <c r="B100" s="2" t="inlineStr"/>
-      <c r="C100" s="2" t="inlineStr"/>
-      <c r="D100" s="2" t="inlineStr"/>
-      <c r="E100" s="2" t="inlineStr"/>
-      <c r="F100" s="2" t="inlineStr"/>
-      <c r="G100" s="2" t="inlineStr"/>
-    </row>
-    <row r="101">
-      <c r="A101" s="2" t="n">
-        <v>100</v>
-      </c>
-      <c r="B101" s="2" t="inlineStr"/>
-      <c r="C101" s="2" t="inlineStr"/>
-      <c r="D101" s="2" t="inlineStr"/>
-      <c r="E101" s="2" t="inlineStr"/>
-      <c r="F101" s="2" t="inlineStr"/>
-      <c r="G101" s="2" t="inlineStr"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G101"/>
+  <autoFilter ref="A1:G21"/>
   <dataValidations count="1">
-    <dataValidation sqref="E2:E101" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>'List Dataset'!$B$2:$B$21</formula1>
+    <dataValidation sqref="E2:E21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>=DatasetList</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
docs: remove shared notebook column from submissions
</commit_message>
<xml_diff>
--- a/spreadsheet/linear_regression_dataset_spreadsheet.xlsx
+++ b/spreadsheet/linear_regression_dataset_spreadsheet.xlsx
@@ -13,7 +13,7 @@
   <definedNames>
     <definedName name="DatasetList">'List Dataset'!$B$2:$B$21</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'List Dataset'!$A$1:$F$21</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pengumpulan'!$A$1:$G$21</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Pengumpulan'!$A$1:$F$21</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1155,7 +1155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1163,8 +1163,7 @@
     <col width="18" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="42" customWidth="1" min="5" max="5"/>
-    <col width="54" customWidth="1" min="6" max="6"/>
-    <col width="54" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1194,11 +1193,6 @@
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>Link Notebook Colab Shared</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
         <is>
           <t>Link Pengumpulan Peserta</t>
         </is>
@@ -1213,7 +1207,6 @@
       <c r="D2" s="2" t="inlineStr"/>
       <c r="E2" s="6" t="inlineStr"/>
       <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -1224,7 +1217,6 @@
       <c r="D3" s="2" t="inlineStr"/>
       <c r="E3" s="6" t="inlineStr"/>
       <c r="F3" s="2" t="inlineStr"/>
-      <c r="G3" s="2" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -1235,7 +1227,6 @@
       <c r="D4" s="2" t="inlineStr"/>
       <c r="E4" s="6" t="inlineStr"/>
       <c r="F4" s="2" t="inlineStr"/>
-      <c r="G4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1246,7 +1237,6 @@
       <c r="D5" s="2" t="inlineStr"/>
       <c r="E5" s="6" t="inlineStr"/>
       <c r="F5" s="2" t="inlineStr"/>
-      <c r="G5" s="2" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -1257,7 +1247,6 @@
       <c r="D6" s="2" t="inlineStr"/>
       <c r="E6" s="6" t="inlineStr"/>
       <c r="F6" s="2" t="inlineStr"/>
-      <c r="G6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -1268,7 +1257,6 @@
       <c r="D7" s="2" t="inlineStr"/>
       <c r="E7" s="6" t="inlineStr"/>
       <c r="F7" s="2" t="inlineStr"/>
-      <c r="G7" s="2" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1279,7 +1267,6 @@
       <c r="D8" s="2" t="inlineStr"/>
       <c r="E8" s="6" t="inlineStr"/>
       <c r="F8" s="2" t="inlineStr"/>
-      <c r="G8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -1290,7 +1277,6 @@
       <c r="D9" s="2" t="inlineStr"/>
       <c r="E9" s="6" t="inlineStr"/>
       <c r="F9" s="2" t="inlineStr"/>
-      <c r="G9" s="2" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -1301,7 +1287,6 @@
       <c r="D10" s="2" t="inlineStr"/>
       <c r="E10" s="6" t="inlineStr"/>
       <c r="F10" s="2" t="inlineStr"/>
-      <c r="G10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1312,7 +1297,6 @@
       <c r="D11" s="2" t="inlineStr"/>
       <c r="E11" s="6" t="inlineStr"/>
       <c r="F11" s="2" t="inlineStr"/>
-      <c r="G11" s="2" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -1323,7 +1307,6 @@
       <c r="D12" s="2" t="inlineStr"/>
       <c r="E12" s="6" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
-      <c r="G12" s="2" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -1334,7 +1317,6 @@
       <c r="D13" s="2" t="inlineStr"/>
       <c r="E13" s="6" t="inlineStr"/>
       <c r="F13" s="2" t="inlineStr"/>
-      <c r="G13" s="2" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1345,7 +1327,6 @@
       <c r="D14" s="2" t="inlineStr"/>
       <c r="E14" s="6" t="inlineStr"/>
       <c r="F14" s="2" t="inlineStr"/>
-      <c r="G14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1356,7 +1337,6 @@
       <c r="D15" s="2" t="inlineStr"/>
       <c r="E15" s="6" t="inlineStr"/>
       <c r="F15" s="2" t="inlineStr"/>
-      <c r="G15" s="2" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1367,7 +1347,6 @@
       <c r="D16" s="2" t="inlineStr"/>
       <c r="E16" s="6" t="inlineStr"/>
       <c r="F16" s="2" t="inlineStr"/>
-      <c r="G16" s="2" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1378,7 +1357,6 @@
       <c r="D17" s="2" t="inlineStr"/>
       <c r="E17" s="6" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
-      <c r="G17" s="2" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1389,7 +1367,6 @@
       <c r="D18" s="2" t="inlineStr"/>
       <c r="E18" s="6" t="inlineStr"/>
       <c r="F18" s="2" t="inlineStr"/>
-      <c r="G18" s="2" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1400,7 +1377,6 @@
       <c r="D19" s="2" t="inlineStr"/>
       <c r="E19" s="6" t="inlineStr"/>
       <c r="F19" s="2" t="inlineStr"/>
-      <c r="G19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1411,7 +1387,6 @@
       <c r="D20" s="2" t="inlineStr"/>
       <c r="E20" s="6" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
-      <c r="G20" s="2" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1422,10 +1397,9 @@
       <c r="D21" s="2" t="inlineStr"/>
       <c r="E21" s="6" t="inlineStr"/>
       <c r="F21" s="2" t="inlineStr"/>
-      <c r="G21" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G21"/>
+  <autoFilter ref="A1:F21"/>
   <dataValidations count="1">
     <dataValidation sqref="E2:E21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>=DatasetList</formula1>

</xml_diff>